<commit_message>
Excel - Functions,Statergic logics,conditional formating
This Excel file the complete beginner working /analysis on data set have performed for eg - Raw data obeservations/scheduling ,budgeting etc
</commit_message>
<xml_diff>
--- a/TASK 2.xlsx
+++ b/TASK 2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9a1e314b52a5af4/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9a1e314b52a5af4/Desktop/DA Assignments/Assignment 1 - ENTRI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="8_{30E95DAD-B360-4E1F-BD01-3690D64A8049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7F24093-D230-449A-8005-E8DCC5F437E4}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{30E95DAD-B360-4E1F-BD01-3690D64A8049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91EBB198-B95E-450E-8785-4EBD0992384A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Dataset!$A$1:$K$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Dataset!$A$1:$K$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3876,5 +3877,6 @@
   </sheetData>
   <autoFilter ref="A1:K36" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="65" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>